<commit_message>
Update feature status: 27/34 done (Phase A + analytical mode completed)
Phase A completed: #1 (core question), #2 (sub-questions), #4 (axes), #5 (research plan)
Analytical mode completed: #44 (synthesis adapts by dispute type)
Score: 22/34 → 27/34 done, 7 partial → 3 partial, 6 not started → 4 not started

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v1_Pruning_Scorecard.xlsx
+++ b/v1_Pruning_Scorecard.xlsx
@@ -881,7 +881,7 @@
       <c r="L4" s="18" t="n"/>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL → Phase A planned (ADR-0006)</t>
+          <t>DONE — QuestionDecomposition.core_question (Phase A)</t>
         </is>
       </c>
       <c r="N4" s="6" t="n"/>
@@ -952,7 +952,7 @@
       <c r="L5" s="18" t="n"/>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>NOT STARTED → Phase A planned (ADR-0006)</t>
+          <t>DONE — SubQuestion with typed decomposition (Phase A, ADR-0006)</t>
         </is>
       </c>
       <c r="N5" s="6" t="n"/>
@@ -1082,7 +1082,7 @@
       <c r="L7" s="26" t="n"/>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>NOT STARTED → Phase A planned (ADR-0006)</t>
+          <t>DONE — QuestionDecomposition.optimization_axes (Phase A)</t>
         </is>
       </c>
       <c r="N7" s="6" t="n"/>
@@ -1145,7 +1145,7 @@
       <c r="L8" s="28" t="n"/>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL → Phase A planned (ADR-0006)</t>
+          <t>DONE — QuestionDecomposition.research_plan + falsification_targets (Phase A)</t>
         </is>
       </c>
       <c r="N8" s="6" t="n"/>
@@ -4032,7 +4032,7 @@
       <c r="L61" s="26" t="n"/>
       <c r="M61" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL → Phase E planned</t>
+          <t>DONE — synthesis_mode config: analytical vs grounded</t>
         </is>
       </c>
       <c r="N61" s="6" t="n"/>

</xml_diff>

<commit_message>
Final scorecard audit: 42 DONE, 4 SKIP, 3 CUT, 3 DEFER→SKIP
Divergences from original plan:
- #3 CUT→DONE: ambiguous terms added (Brian wanted this)
- #38 CUT→DONE: position shuffling added (Brian disagreed with CUT)
- #8,9,10,12 DEFER→DONE: decomposition validation promoted
- #30 DEFER→DONE: evidence leakage check promoted
- #11,14,17,43 DEFER→SKIP: confirmed not worth building

42/52 features implemented. 4 intentionally skipped. 3 cut. 3 deferred→skipped.
Full scorecard complete.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v1_Pruning_Scorecard.xlsx
+++ b/v1_Pruning_Scorecard.xlsx
@@ -1023,7 +1023,7 @@
       <c r="L6" s="25" t="n"/>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>CUT</t>
+          <t>DONE — AmbiguousTerm schema, decomposition identifies and passes to analysts</t>
         </is>
       </c>
       <c r="N6" s="6" t="n"/>
@@ -1412,7 +1412,7 @@
       <c r="L13" s="26" t="n"/>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>DONE — DecompositionValidation checks coverage gaps</t>
         </is>
       </c>
       <c r="N13" s="6" t="n"/>
@@ -1471,7 +1471,7 @@
       <c r="L14" s="26" t="n"/>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>DONE — DecompositionValidation checks directional bias</t>
         </is>
       </c>
       <c r="N14" s="6" t="n"/>
@@ -1530,7 +1530,7 @@
       <c r="L15" s="26" t="n"/>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>DONE — DecompositionValidation checks granularity (broad/narrow/redundant)</t>
         </is>
       </c>
       <c r="N15" s="6" t="n"/>
@@ -1589,7 +1589,7 @@
       <c r="L16" s="26" t="n"/>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>SKIP — falsification targets exist but quality validation deferred (low value)</t>
         </is>
       </c>
       <c r="N16" s="6" t="n"/>
@@ -1648,7 +1648,7 @@
       <c r="L17" s="26" t="n"/>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>DONE — proceed/revise verdict with one retry on revise</t>
         </is>
       </c>
       <c r="N17" s="6" t="n"/>
@@ -1832,7 +1832,7 @@
       <c r="L21" s="26" t="n"/>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>SKIP — Reddit/Grok API is a separate search provider, not pipeline feature</t>
         </is>
       </c>
       <c r="N21" s="6" t="n"/>
@@ -2045,7 +2045,7 @@
       <c r="L24" s="18" t="n"/>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>SKIP — Brian said "I wouldnt even try this"</t>
         </is>
       </c>
       <c r="N24" s="6" t="n"/>
@@ -2611,7 +2611,7 @@
       <c r="L34" s="26" t="n"/>
       <c r="M34" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL → Phase E planned</t>
+          <t>DONE — counterarguments min_length=1 in AnalystRun schema</t>
         </is>
       </c>
       <c r="N34" s="6" t="n"/>
@@ -2988,7 +2988,7 @@
       <c r="L41" s="26" t="n"/>
       <c r="M41" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>DONE — URL regex scan on analyst outputs, warns on leakage</t>
         </is>
       </c>
       <c r="N41" s="6" t="n"/>
@@ -3546,7 +3546,7 @@
       <c r="L51" s="26" t="n"/>
       <c r="M51" s="6" t="inlineStr">
         <is>
-          <t>CUT</t>
+          <t>DONE — random.shuffle(claims) with fixed seed per dispute in arbitration</t>
         </is>
       </c>
       <c r="N51" s="6" t="n"/>
@@ -3914,7 +3914,7 @@
       <c r="L59" s="26" t="n"/>
       <c r="M59" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL → Phase E planned</t>
+          <t>DONE — compress.py priority-based compression when over threshold</t>
         </is>
       </c>
       <c r="N59" s="6" t="n"/>
@@ -3973,7 +3973,7 @@
       <c r="L60" s="26" t="n"/>
       <c r="M60" s="6" t="inlineStr">
         <is>
-          <t>DEFERRED (tested: no self-preference bias)</t>
+          <t>SKIP — tested with 2 judge models, no self-preference detected</t>
         </is>
       </c>
       <c r="N60" s="6" t="n"/>
@@ -4464,7 +4464,7 @@
       <c r="L69" s="17" t="n"/>
       <c r="M69" s="6" t="inlineStr">
         <is>
-          <t>NOT STARTED → Phase C planned</t>
+          <t>DONE — model_fallbacks config + get_fallback_models() on all 10 call sites</t>
         </is>
       </c>
       <c r="N69" s="6" t="n"/>

</xml_diff>

<commit_message>
Fix stale Excel entries: #15,18,19,40,41 updated to DONE
These were implemented but Excel still showed old status (PARTIAL/NOT STARTED).
Accurate count: 47 DONE, 4 SKIP, 1 CUT = 52 total.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v1_Pruning_Scorecard.xlsx
+++ b/v1_Pruning_Scorecard.xlsx
@@ -1903,7 +1903,7 @@
       <c r="L22" s="25" t="n"/>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL → Phase B planned</t>
+          <t>DONE — source_quality.py LLM batch scoring (authoritative/reliable/unknown/unreliable)</t>
         </is>
       </c>
       <c r="N22" s="6" t="n"/>
@@ -2116,7 +2116,7 @@
       <c r="L25" s="18" t="n"/>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>NOT STARTED → Phase B planned</t>
+          <t>DONE — compress.py priority-based compression preserving authoritative + diverse</t>
         </is>
       </c>
       <c r="N25" s="6" t="n"/>
@@ -2175,7 +2175,7 @@
       <c r="L26" s="26" t="n"/>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL → Phase B planned</t>
+          <t>DONE — per-sub-question evidence sufficiency check, flags gaps for &lt;2 items</t>
         </is>
       </c>
       <c r="N26" s="6" t="n"/>
@@ -3730,7 +3730,7 @@
       <c r="L55" s="26" t="n"/>
       <c r="M55" s="6" t="inlineStr">
         <is>
-          <t>NOT STARTED → Phase D planned</t>
+          <t>DONE — filters preference/ambiguity disputes, prompts user in TTY mode</t>
         </is>
       </c>
       <c r="N55" s="6" t="n"/>
@@ -3789,7 +3789,7 @@
       <c r="L56" s="26" t="n"/>
       <c r="M56" s="6" t="inlineStr">
         <is>
-          <t>NOT STARTED → Phase D planned</t>
+          <t>DONE — max 2 structured questions with defaults, auto-skip non-interactive</t>
         </is>
       </c>
       <c r="N56" s="6" t="n"/>

</xml_diff>

<commit_message>
Add Where Implemented + Implementation Notes columns to scorecard
Col 14: file paths where each feature is implemented
Col 15: concise commentary on the implementation approach

All 52 rows populated with specific file locations and notes.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v1_Pruning_Scorecard.xlsx
+++ b/v1_Pruning_Scorecard.xlsx
@@ -747,8 +747,16 @@
           <t>Implementation Status (2026-03-23)</t>
         </is>
       </c>
-      <c r="N1" s="6" t="n"/>
-      <c r="O1" s="6" t="n"/>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Where Implemented</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>Implementation Notes</t>
+        </is>
+      </c>
       <c r="P1" s="6" t="n"/>
       <c r="Q1" s="6" t="n"/>
       <c r="R1" s="6" t="n"/>
@@ -884,8 +892,16 @@
           <t>DONE — QuestionDecomposition.core_question (Phase A)</t>
         </is>
       </c>
-      <c r="N4" s="6" t="n"/>
-      <c r="O4" s="6" t="n"/>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, models.py</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>QuestionDecomposition.core_question via LLM structured output</t>
+        </is>
+      </c>
       <c r="P4" s="6" t="n"/>
       <c r="Q4" s="6" t="n"/>
       <c r="R4" s="6" t="n"/>
@@ -955,8 +971,16 @@
           <t>DONE — SubQuestion with typed decomposition (Phase A, ADR-0006)</t>
         </is>
       </c>
-      <c r="N5" s="6" t="n"/>
-      <c r="O5" s="6" t="n"/>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, models.py</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>SubQuestion with typed enum (factual/causal/comparative/evaluative/scope) + falsification_target. ADR-0006.</t>
+        </is>
+      </c>
       <c r="P5" s="6" t="n"/>
       <c r="Q5" s="6" t="n"/>
       <c r="R5" s="6" t="n"/>
@@ -1026,8 +1050,16 @@
           <t>DONE — AmbiguousTerm schema, decomposition identifies and passes to analysts</t>
         </is>
       </c>
-      <c r="N6" s="6" t="n"/>
-      <c r="O6" s="6" t="n"/>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, models.py, analyst.yaml</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>AmbiguousTerm schema. Decomposition identifies, analysts receive as context. Was CUT, Brian disagreed.</t>
+        </is>
+      </c>
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="6" t="n"/>
       <c r="R6" s="6" t="n"/>
@@ -1085,8 +1117,16 @@
           <t>DONE — QuestionDecomposition.optimization_axes (Phase A)</t>
         </is>
       </c>
-      <c r="N7" s="6" t="n"/>
-      <c r="O7" s="6" t="n"/>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, models.py, long_report.yaml</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>optimization_axes field. Passed to synthesis as organizing framework for key distinctions.</t>
+        </is>
+      </c>
       <c r="P7" s="6" t="n"/>
       <c r="Q7" s="6" t="n"/>
       <c r="R7" s="6" t="n"/>
@@ -1148,8 +1188,16 @@
           <t>DONE — QuestionDecomposition.research_plan + falsification_targets (Phase A)</t>
         </is>
       </c>
-      <c r="N8" s="6" t="n"/>
-      <c r="O8" s="6" t="n"/>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, models.py</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>research_plan field + per-SQ falsification_target drives counterfactual search queries.</t>
+        </is>
+      </c>
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="6" t="n"/>
@@ -1219,8 +1267,16 @@
           <t>CUT</t>
         </is>
       </c>
-      <c r="N9" s="6" t="n"/>
-      <c r="O9" s="6" t="n"/>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>CUT — complexity level doesnt control anything in the pipeline.</t>
+        </is>
+      </c>
       <c r="P9" s="6" t="n"/>
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="6" t="n"/>
@@ -1290,8 +1346,16 @@
           <t>DONE — PhaseTrace.output_summary</t>
         </is>
       </c>
-      <c r="N10" s="6" t="n"/>
-      <c r="O10" s="6" t="n"/>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>engine.py, models.py</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>PhaseTrace.output_summary written per phase in engine.py.</t>
+        </is>
+      </c>
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="6" t="n"/>
@@ -1415,8 +1479,16 @@
           <t>DONE — DecompositionValidation checks coverage gaps</t>
         </is>
       </c>
-      <c r="N13" s="6" t="n"/>
-      <c r="O13" s="6" t="n"/>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, validate_decomposition.yaml</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>DecompositionValidation.coverage_ok + coverage_gaps. Single LLM call.</t>
+        </is>
+      </c>
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
       <c r="R13" s="6" t="n"/>
@@ -1474,8 +1546,16 @@
           <t>DONE — DecompositionValidation checks directional bias</t>
         </is>
       </c>
-      <c r="N14" s="6" t="n"/>
-      <c r="O14" s="6" t="n"/>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, validate_decomposition.yaml</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>DecompositionValidation.bias_flags. Same call as #8.</t>
+        </is>
+      </c>
       <c r="P14" s="6" t="n"/>
       <c r="Q14" s="6" t="n"/>
       <c r="R14" s="6" t="n"/>
@@ -1533,8 +1613,16 @@
           <t>DONE — DecompositionValidation checks granularity (broad/narrow/redundant)</t>
         </is>
       </c>
-      <c r="N15" s="6" t="n"/>
-      <c r="O15" s="6" t="n"/>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py, validate_decomposition.yaml</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>DecompositionValidation.granularity_issues. Same call as #8-9.</t>
+        </is>
+      </c>
       <c r="P15" s="6" t="n"/>
       <c r="Q15" s="6" t="n"/>
       <c r="R15" s="6" t="n"/>
@@ -1592,8 +1680,16 @@
           <t>SKIP — falsification targets exist but quality validation deferred (low value)</t>
         </is>
       </c>
-      <c r="N16" s="6" t="n"/>
-      <c r="O16" s="6" t="n"/>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>SKIP — falsification targets exist but validating their quality is meta-validation with unclear value.</t>
+        </is>
+      </c>
       <c r="P16" s="6" t="n"/>
       <c r="Q16" s="6" t="n"/>
       <c r="R16" s="6" t="n"/>
@@ -1651,8 +1747,16 @@
           <t>DONE — proceed/revise verdict with one retry on revise</t>
         </is>
       </c>
-      <c r="N17" s="6" t="n"/>
-      <c r="O17" s="6" t="n"/>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>decompose.py</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>proceed/revise verdict with one retry. decompose_with_validation() re-runs on revise.</t>
+        </is>
+      </c>
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="6" t="n"/>
       <c r="R17" s="6" t="n"/>
@@ -1776,8 +1880,16 @@
           <t>DONE — generate_search_queries()</t>
         </is>
       </c>
-      <c r="N20" s="6" t="n"/>
-      <c r="O20" s="6" t="n"/>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>collect.py</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>generate_search_queries() per sub-question. Parallel via asyncio.gather.</t>
+        </is>
+      </c>
       <c r="P20" s="6" t="n"/>
       <c r="Q20" s="6" t="n"/>
       <c r="R20" s="6" t="n"/>
@@ -1835,8 +1947,16 @@
           <t>SKIP — Reddit/Grok API is a separate search provider, not pipeline feature</t>
         </is>
       </c>
-      <c r="N21" s="6" t="n"/>
-      <c r="O21" s="6" t="n"/>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>SKIP — separate search provider integration, not a pipeline feature.</t>
+        </is>
+      </c>
       <c r="P21" s="6" t="n"/>
       <c r="Q21" s="6" t="n"/>
       <c r="R21" s="6" t="n"/>
@@ -1906,8 +2026,16 @@
           <t>DONE — source_quality.py LLM batch scoring (authoritative/reliable/unknown/unreliable)</t>
         </is>
       </c>
-      <c r="N22" s="6" t="n"/>
-      <c r="O22" s="6" t="n"/>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>source_quality.py</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>LLM batch scoring: authoritative/reliable/unknown/unreliable. Inline prompt (tech debt).</t>
+        </is>
+      </c>
       <c r="P22" s="6" t="n"/>
       <c r="Q22" s="6" t="n"/>
       <c r="R22" s="6" t="n"/>
@@ -1977,8 +2105,16 @@
           <t>DONE — fetch_page() extraction</t>
         </is>
       </c>
-      <c r="N23" s="6" t="n"/>
-      <c r="O23" s="6" t="n"/>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>collect.py, tools/fetch_page.py</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>fetch_page extracts key_section + notes. Jina Reader fallback for 403s.</t>
+        </is>
+      </c>
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="6" t="n"/>
       <c r="R23" s="6" t="n"/>
@@ -2048,8 +2184,16 @@
           <t>SKIP — Brian said "I wouldnt even try this"</t>
         </is>
       </c>
-      <c r="N24" s="6" t="n"/>
-      <c r="O24" s="6" t="n"/>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>SKIP — Brian: "I wouldnt even try this."</t>
+        </is>
+      </c>
       <c r="P24" s="6" t="n"/>
       <c r="Q24" s="6" t="n"/>
       <c r="R24" s="6" t="n"/>
@@ -2119,8 +2263,16 @@
           <t>DONE — compress.py priority-based compression preserving authoritative + diverse</t>
         </is>
       </c>
-      <c r="N25" s="6" t="n"/>
-      <c r="O25" s="6" t="n"/>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>compress.py, engine.py</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>Priority-based compression: authoritative first, sub-question coverage, diversity. Configurable threshold.</t>
+        </is>
+      </c>
       <c r="P25" s="6" t="n"/>
       <c r="Q25" s="6" t="n"/>
       <c r="R25" s="6" t="n"/>
@@ -2178,8 +2330,16 @@
           <t>DONE — per-sub-question evidence sufficiency check, flags gaps for &lt;2 items</t>
         </is>
       </c>
-      <c r="N26" s="6" t="n"/>
-      <c r="O26" s="6" t="n"/>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>engine.py, models.py</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>EvidenceItem.sub_question_id tracks origin. engine.py checks coverage per SQ, flags gaps.</t>
+        </is>
+      </c>
       <c r="P26" s="6" t="n"/>
       <c r="Q26" s="6" t="n"/>
       <c r="R26" s="6" t="n"/>
@@ -2241,8 +2401,16 @@
           <t>DONE — config num_queries/max_sources</t>
         </is>
       </c>
-      <c r="N27" s="6" t="n"/>
-      <c r="O27" s="6" t="n"/>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>config.yaml, collect.py</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>num_queries and max_sources in config. Depth profiles override for deep/thorough.</t>
+        </is>
+      </c>
       <c r="P27" s="6" t="n"/>
       <c r="Q27" s="6" t="n"/>
       <c r="R27" s="6" t="n"/>
@@ -2366,8 +2534,16 @@
           <t>DONE — run_analysts() cross-family + frames</t>
         </is>
       </c>
-      <c r="N30" s="6" t="n"/>
-      <c r="O30" s="6" t="n"/>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>analysts.py, config.yaml</t>
+        </is>
+      </c>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>run_analysts() with 3 cross-family models + 3 distinct frames. asyncio.gather parallel.</t>
+        </is>
+      </c>
       <c r="P30" s="6" t="n"/>
       <c r="Q30" s="6" t="n"/>
       <c r="R30" s="6" t="n"/>
@@ -2425,8 +2601,16 @@
           <t>DONE — AnalystRun.recommendations</t>
         </is>
       </c>
-      <c r="N31" s="6" t="n"/>
-      <c r="O31" s="6" t="n"/>
+      <c r="N31" s="6" t="inlineStr">
+        <is>
+          <t>models.py, analyst.yaml</t>
+        </is>
+      </c>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>AnalystRun.recommendations is a required schema field.</t>
+        </is>
+      </c>
       <c r="P31" s="6" t="n"/>
       <c r="Q31" s="6" t="n"/>
       <c r="R31" s="6" t="n"/>
@@ -2496,8 +2680,16 @@
           <t>DONE — RawClaim.evidence_ids + hallucination stripping</t>
         </is>
       </c>
-      <c r="N32" s="6" t="n"/>
-      <c r="O32" s="6" t="n"/>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>models.py, canonicalize.py</t>
+        </is>
+      </c>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
+          <t>RawClaim.evidence_ids required. Hallucinated IDs stripped in extract_raw_claims().</t>
+        </is>
+      </c>
       <c r="P32" s="6" t="n"/>
       <c r="Q32" s="6" t="n"/>
       <c r="R32" s="6" t="n"/>
@@ -2555,8 +2747,16 @@
           <t>DONE — AnalystRun.assumptions</t>
         </is>
       </c>
-      <c r="N33" s="6" t="n"/>
-      <c r="O33" s="6" t="n"/>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>models.py</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>AnalystRun.assumptions schema field.</t>
+        </is>
+      </c>
       <c r="P33" s="6" t="n"/>
       <c r="Q33" s="6" t="n"/>
       <c r="R33" s="6" t="n"/>
@@ -2614,8 +2814,16 @@
           <t>DONE — counterarguments min_length=1 in AnalystRun schema</t>
         </is>
       </c>
-      <c r="N34" s="6" t="n"/>
-      <c r="O34" s="6" t="n"/>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>models.py</t>
+        </is>
+      </c>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>AnalystRun.counterarguments min_length=1 — schema enforces at least one.</t>
+        </is>
+      </c>
       <c r="P34" s="6" t="n"/>
       <c r="Q34" s="6" t="n"/>
       <c r="R34" s="6" t="n"/>
@@ -2673,8 +2881,16 @@
           <t>DONE — Alpha/Beta/Gamma labels, blind by construction</t>
         </is>
       </c>
-      <c r="N35" s="6" t="n"/>
-      <c r="O35" s="6" t="n"/>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>analysts.py</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>Labels Alpha/Beta/Gamma. Analysts never see each others outputs by construction.</t>
+        </is>
+      </c>
       <c r="P35" s="6" t="n"/>
       <c r="Q35" s="6" t="n"/>
       <c r="R35" s="6" t="n"/>
@@ -2810,8 +3026,16 @@
           <t>DONE — extract_raw_claims()</t>
         </is>
       </c>
-      <c r="N38" s="6" t="n"/>
-      <c r="O38" s="6" t="n"/>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>canonicalize.py</t>
+        </is>
+      </c>
+      <c r="O38" s="6" t="inlineStr">
+        <is>
+          <t>extract_raw_claims() — simple Python extraction from analyst runs, no LLM.</t>
+        </is>
+      </c>
       <c r="P38" s="6" t="n"/>
       <c r="Q38" s="6" t="n"/>
       <c r="R38" s="6" t="n"/>
@@ -2881,8 +3105,16 @@
           <t>DONE — deduplicate_claims() via LLM</t>
         </is>
       </c>
-      <c r="N39" s="6" t="n"/>
-      <c r="O39" s="6" t="n"/>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>canonicalize.py, dedup.yaml</t>
+        </is>
+      </c>
+      <c r="O39" s="6" t="inlineStr">
+        <is>
+          <t>deduplicate_claims() via LLM grouping. Fallback: 1:1 promotion if 0 groups.</t>
+        </is>
+      </c>
       <c r="P39" s="6" t="n"/>
       <c r="Q39" s="6" t="n"/>
       <c r="R39" s="6" t="n"/>
@@ -2936,8 +3168,16 @@
           <t>DONE — C- prefix IDs, evidence_ids propagated</t>
         </is>
       </c>
-      <c r="N40" s="6" t="n"/>
-      <c r="O40" s="6" t="n"/>
+      <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>models.py</t>
+        </is>
+      </c>
+      <c r="O40" s="6" t="inlineStr">
+        <is>
+          <t>C- prefix IDs via _make_id(). evidence_ids propagated through dedup.</t>
+        </is>
+      </c>
       <c r="P40" s="6" t="n"/>
       <c r="Q40" s="6" t="n"/>
       <c r="R40" s="6" t="n"/>
@@ -2991,8 +3231,16 @@
           <t>DONE — URL regex scan on analyst outputs, warns on leakage</t>
         </is>
       </c>
-      <c r="N41" s="6" t="n"/>
-      <c r="O41" s="6" t="n"/>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>engine.py</t>
+        </is>
+      </c>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>URL regex scan on analyst claims + summary after Phase 2. Emits PipelineWarning.</t>
+        </is>
+      </c>
       <c r="P41" s="6" t="n"/>
       <c r="Q41" s="6" t="n"/>
       <c r="R41" s="6" t="n"/>
@@ -3062,8 +3310,16 @@
           <t>DONE — detect_disputes() 4 types</t>
         </is>
       </c>
-      <c r="N42" s="6" t="n"/>
-      <c r="O42" s="6" t="n"/>
+      <c r="N42" s="6" t="inlineStr">
+        <is>
+          <t>canonicalize.py, dispute_classify.yaml</t>
+        </is>
+      </c>
+      <c r="O42" s="6" t="inlineStr">
+        <is>
+          <t>detect_disputes() with 4 types: factual_conflict, interpretive_conflict, preference_conflict, ambiguity.</t>
+        </is>
+      </c>
       <c r="P42" s="6" t="n"/>
       <c r="Q42" s="6" t="n"/>
       <c r="R42" s="6" t="n"/>
@@ -3117,8 +3373,16 @@
           <t>DONE — severity classification (ADR-0005 fix)</t>
         </is>
       </c>
-      <c r="N43" s="6" t="n"/>
-      <c r="O43" s="6" t="n"/>
+      <c r="N43" s="6" t="inlineStr">
+        <is>
+          <t>canonicalize.py, dispute_classify.yaml</t>
+        </is>
+      </c>
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>Severity in schema Field(description) with guidance. Gemini-2.5-flash model (not lite).</t>
+        </is>
+      </c>
       <c r="P43" s="6" t="n"/>
       <c r="Q43" s="6" t="n"/>
       <c r="R43" s="6" t="n"/>
@@ -3188,8 +3452,16 @@
           <t>DONE — DISPUTE_ROUTING code-owned table</t>
         </is>
       </c>
-      <c r="N44" s="6" t="n"/>
-      <c r="O44" s="6" t="n"/>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>models.py</t>
+        </is>
+      </c>
+      <c r="O44" s="6" t="inlineStr">
+        <is>
+          <t>DISPUTE_ROUTING dict: code-owned mapping of dispute_type → route.</t>
+        </is>
+      </c>
       <c r="P44" s="6" t="n"/>
       <c r="Q44" s="6" t="n"/>
       <c r="R44" s="6" t="n"/>
@@ -3313,8 +3585,16 @@
           <t>DONE — generate_verification_queries()</t>
         </is>
       </c>
-      <c r="N47" s="6" t="n"/>
-      <c r="O47" s="6" t="n"/>
+      <c r="N47" s="6" t="inlineStr">
+        <is>
+          <t>verify.py, verification_queries.yaml</t>
+        </is>
+      </c>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>generate_verification_queries() produces counterfactual search queries per dispute.</t>
+        </is>
+      </c>
       <c r="P47" s="6" t="n"/>
       <c r="Q47" s="6" t="n"/>
       <c r="R47" s="6" t="n"/>
@@ -3372,8 +3652,16 @@
           <t>DONE — Brave Search fresh evidence</t>
         </is>
       </c>
-      <c r="N48" s="6" t="n"/>
-      <c r="O48" s="6" t="n"/>
+      <c r="N48" s="6" t="inlineStr">
+        <is>
+          <t>verify.py, tools/brave_search.py</t>
+        </is>
+      </c>
+      <c r="O48" s="6" t="inlineStr">
+        <is>
+          <t>Fresh evidence fetched via Brave Search during arbitration.</t>
+        </is>
+      </c>
       <c r="P48" s="6" t="n"/>
       <c r="Q48" s="6" t="n"/>
       <c r="R48" s="6" t="n"/>
@@ -3431,8 +3719,16 @@
           <t>DONE — arbitrate_dispute() structured</t>
         </is>
       </c>
-      <c r="N49" s="6" t="n"/>
-      <c r="O49" s="6" t="n"/>
+      <c r="N49" s="6" t="inlineStr">
+        <is>
+          <t>verify.py, arbitration.yaml</t>
+        </is>
+      </c>
+      <c r="O49" s="6" t="inlineStr">
+        <is>
+          <t>arbitrate_dispute() returns typed ArbitrationResult. Claims shuffled per #38.</t>
+        </is>
+      </c>
       <c r="P49" s="6" t="n"/>
       <c r="Q49" s="6" t="n"/>
       <c r="R49" s="6" t="n"/>
@@ -3490,8 +3786,16 @@
           <t>DONE — ArbitrationResult.claim_updates</t>
         </is>
       </c>
-      <c r="N50" s="6" t="n"/>
-      <c r="O50" s="6" t="n"/>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>verify.py</t>
+        </is>
+      </c>
+      <c r="O50" s="6" t="inlineStr">
+        <is>
+          <t>ArbitrationResult.claim_updates applied to ledger. ADR-0004 invariant enforced.</t>
+        </is>
+      </c>
       <c r="P50" s="6" t="n"/>
       <c r="Q50" s="6" t="n"/>
       <c r="R50" s="6" t="n"/>
@@ -3549,8 +3853,16 @@
           <t>DONE — random.shuffle(claims) with fixed seed per dispute in arbitration</t>
         </is>
       </c>
-      <c r="N51" s="6" t="n"/>
-      <c r="O51" s="6" t="n"/>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>verify.py</t>
+        </is>
+      </c>
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>random.shuffle(claims) with fixed seed (dispute.id) before arbitration. Was CUT, Brian disagreed.</t>
+        </is>
+      </c>
       <c r="P51" s="6" t="n"/>
       <c r="Q51" s="6" t="n"/>
       <c r="R51" s="6" t="n"/>
@@ -3608,8 +3920,16 @@
           <t>DONE — config max_disputes/max_turns</t>
         </is>
       </c>
-      <c r="N52" s="6" t="n"/>
-      <c r="O52" s="6" t="n"/>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>config.yaml</t>
+        </is>
+      </c>
+      <c r="O52" s="6" t="inlineStr">
+        <is>
+          <t>max_disputes and max_turns in budgets config.</t>
+        </is>
+      </c>
       <c r="P52" s="6" t="n"/>
       <c r="Q52" s="6" t="n"/>
       <c r="R52" s="6" t="n"/>
@@ -3733,8 +4053,16 @@
           <t>DONE — filters preference/ambiguity disputes, prompts user in TTY mode</t>
         </is>
       </c>
-      <c r="N55" s="6" t="n"/>
-      <c r="O55" s="6" t="n"/>
+      <c r="N55" s="6" t="inlineStr">
+        <is>
+          <t>engine.py</t>
+        </is>
+      </c>
+      <c r="O55" s="6" t="inlineStr">
+        <is>
+          <t>Filters preference/ambiguity disputes after classification. Prompts user if TTY.</t>
+        </is>
+      </c>
       <c r="P55" s="6" t="n"/>
       <c r="Q55" s="6" t="n"/>
       <c r="R55" s="6" t="n"/>
@@ -3792,8 +4120,16 @@
           <t>DONE — max 2 structured questions with defaults, auto-skip non-interactive</t>
         </is>
       </c>
-      <c r="N56" s="6" t="n"/>
-      <c r="O56" s="6" t="n"/>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>engine.py</t>
+        </is>
+      </c>
+      <c r="O56" s="6" t="inlineStr">
+        <is>
+          <t>Max 2 questions. input() with auto-skip on non-TTY. User guidance in dispute.resolution_summary.</t>
+        </is>
+      </c>
       <c r="P56" s="6" t="n"/>
       <c r="Q56" s="6" t="n"/>
       <c r="R56" s="6" t="n"/>
@@ -3917,8 +4253,16 @@
           <t>DONE — compress.py priority-based compression when over threshold</t>
         </is>
       </c>
-      <c r="N59" s="6" t="n"/>
-      <c r="O59" s="6" t="n"/>
+      <c r="N59" s="6" t="inlineStr">
+        <is>
+          <t>compress.py, config.yaml</t>
+        </is>
+      </c>
+      <c r="O59" s="6" t="inlineStr">
+        <is>
+          <t>compress_evidence() with configurable threshold. Depth profiles scale it.</t>
+        </is>
+      </c>
       <c r="P59" s="6" t="n"/>
       <c r="Q59" s="6" t="n"/>
       <c r="R59" s="6" t="n"/>
@@ -3976,8 +4320,16 @@
           <t>SKIP — tested with 2 judge models, no self-preference detected</t>
         </is>
       </c>
-      <c r="N60" s="6" t="n"/>
-      <c r="O60" s="6" t="n"/>
+      <c r="N60" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O60" s="6" t="inlineStr">
+        <is>
+          <t>SKIP — tested with 2 judge models (Gemini + GPT-5-nano), no self-preference bias detected.</t>
+        </is>
+      </c>
       <c r="P60" s="6" t="n"/>
       <c r="Q60" s="6" t="n"/>
       <c r="R60" s="6" t="n"/>
@@ -4035,8 +4387,16 @@
           <t>DONE — synthesis_mode config: analytical vs grounded</t>
         </is>
       </c>
-      <c r="N61" s="6" t="n"/>
-      <c r="O61" s="6" t="n"/>
+      <c r="N61" s="6" t="inlineStr">
+        <is>
+          <t>config.yaml, long_report.yaml, export.py</t>
+        </is>
+      </c>
+      <c r="O61" s="6" t="inlineStr">
+        <is>
+          <t>synthesis_mode: analytical (inferences marked) vs grounded (ledger-only). Provenance always in trace.</t>
+        </is>
+      </c>
       <c r="P61" s="6" t="n"/>
       <c r="Q61" s="6" t="n"/>
       <c r="R61" s="6" t="n"/>
@@ -4094,8 +4454,16 @@
           <t>DONE — FinalReport + long report</t>
         </is>
       </c>
-      <c r="N62" s="6" t="n"/>
-      <c r="O62" s="6" t="n"/>
+      <c r="N62" s="6" t="inlineStr">
+        <is>
+          <t>models.py, export.py, long_report.yaml</t>
+        </is>
+      </c>
+      <c r="O62" s="6" t="inlineStr">
+        <is>
+          <t>FinalReport.recommendation + alternatives. Long report has verdict + alternatives sections.</t>
+        </is>
+      </c>
       <c r="P62" s="6" t="n"/>
       <c r="Q62" s="6" t="n"/>
       <c r="R62" s="6" t="n"/>
@@ -4157,8 +4525,16 @@
           <t>DONE — disagreement_summary + alternatives</t>
         </is>
       </c>
-      <c r="N63" s="6" t="n"/>
-      <c r="O63" s="6" t="n"/>
+      <c r="N63" s="6" t="inlineStr">
+        <is>
+          <t>models.py, export.py</t>
+        </is>
+      </c>
+      <c r="O63" s="6" t="inlineStr">
+        <is>
+          <t>FinalReport.disagreement_summary, alternatives, confidence enum.</t>
+        </is>
+      </c>
       <c r="P63" s="6" t="n"/>
       <c r="Q63" s="6" t="n"/>
       <c r="R63" s="6" t="n"/>
@@ -4216,8 +4592,16 @@
           <t>DONE — trace.json + summary.md</t>
         </is>
       </c>
-      <c r="N64" s="6" t="n"/>
-      <c r="O64" s="6" t="n"/>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>export.py</t>
+        </is>
+      </c>
+      <c r="O64" s="6" t="inlineStr">
+        <is>
+          <t>summary.md with cited claims. trace.json = full PipelineState.</t>
+        </is>
+      </c>
       <c r="P64" s="6" t="n"/>
       <c r="Q64" s="6" t="n"/>
       <c r="R64" s="6" t="n"/>
@@ -4275,8 +4659,16 @@
           <t>DONE — validate_grounding() + hallucination stripping</t>
         </is>
       </c>
-      <c r="N65" s="6" t="n"/>
-      <c r="O65" s="6" t="n"/>
+      <c r="N65" s="6" t="inlineStr">
+        <is>
+          <t>export.py</t>
+        </is>
+      </c>
+      <c r="O65" s="6" t="inlineStr">
+        <is>
+          <t>validate_grounding() checks claim/evidence ID resolution. Hallucinated IDs stripped post-parse.</t>
+        </is>
+      </c>
       <c r="P65" s="6" t="n"/>
       <c r="Q65" s="6" t="n"/>
       <c r="R65" s="6" t="n"/>
@@ -4338,8 +4730,16 @@
           <t>DONE — trace.json = PipelineState</t>
         </is>
       </c>
-      <c r="N66" s="6" t="n"/>
-      <c r="O66" s="6" t="n"/>
+      <c r="N66" s="6" t="inlineStr">
+        <is>
+          <t>engine.py, export.py</t>
+        </is>
+      </c>
+      <c r="O66" s="6" t="inlineStr">
+        <is>
+          <t>trace.json written from PipelineState. Partial trace on failure.</t>
+        </is>
+      </c>
       <c r="P66" s="6" t="n"/>
       <c r="Q66" s="6" t="n"/>
       <c r="R66" s="6" t="n"/>
@@ -4467,8 +4867,16 @@
           <t>DONE — model_fallbacks config + get_fallback_models() on all 10 call sites</t>
         </is>
       </c>
-      <c r="N69" s="6" t="n"/>
-      <c r="O69" s="6" t="n"/>
+      <c r="N69" s="6" t="inlineStr">
+        <is>
+          <t>config.py, config.yaml, all call sites</t>
+        </is>
+      </c>
+      <c r="O69" s="6" t="inlineStr">
+        <is>
+          <t>model_fallbacks config + get_fallback_models(). All 10 LLM call sites pass fallback_models kwarg.</t>
+        </is>
+      </c>
       <c r="P69" s="6" t="n"/>
       <c r="Q69" s="6" t="n"/>
       <c r="R69" s="6" t="n"/>
@@ -4526,8 +4934,16 @@
           <t>DONE — analyst_min_successful config</t>
         </is>
       </c>
-      <c r="N70" s="6" t="n"/>
-      <c r="O70" s="6" t="n"/>
+      <c r="N70" s="6" t="inlineStr">
+        <is>
+          <t>analysts.py, config.yaml</t>
+        </is>
+      </c>
+      <c r="O70" s="6" t="inlineStr">
+        <is>
+          <t>analyst_min_successful in budgets. RuntimeError if &lt;2 succeed.</t>
+        </is>
+      </c>
       <c r="P70" s="6" t="n"/>
       <c r="Q70" s="6" t="n"/>
       <c r="R70" s="6" t="n"/>
@@ -4581,8 +4997,16 @@
           <t>DONE — exception handler writes partial trace</t>
         </is>
       </c>
-      <c r="N71" s="6" t="n"/>
-      <c r="O71" s="6" t="n"/>
+      <c r="N71" s="6" t="inlineStr">
+        <is>
+          <t>engine.py</t>
+        </is>
+      </c>
+      <c r="O71" s="6" t="inlineStr">
+        <is>
+          <t>Exception handler writes trace.json with partial state before re-raising.</t>
+        </is>
+      </c>
       <c r="P71" s="6" t="n"/>
       <c r="Q71" s="6" t="n"/>
       <c r="R71" s="6" t="n"/>

</xml_diff>